<commit_message>
Updated CRM VTIGER CODES
</commit_message>
<xml_diff>
--- a/Crm-Vtiger/src/test/resources/PD.xlsx
+++ b/Crm-Vtiger/src/test/resources/PD.xlsx
@@ -4,17 +4,18 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Leads" sheetId="1" r:id="rId1"/>
+    <sheet name="opportunities" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="242">
   <si>
     <t>Phone</t>
   </si>
@@ -545,13 +546,208 @@
   </si>
   <si>
     <t>Interested in learning about available service plans.</t>
+  </si>
+  <si>
+    <t>Opportunity Name</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Expected Close Date</t>
+  </si>
+  <si>
+    <t>Next Step</t>
+  </si>
+  <si>
+    <t>Probability (%)</t>
+  </si>
+  <si>
+    <t>Website Redesign - BluePeak</t>
+  </si>
+  <si>
+    <t>Send proposal</t>
+  </si>
+  <si>
+    <t>Potential website redesign for BluePeak Retail.</t>
+  </si>
+  <si>
+    <t>CRM Implementation - Northstar</t>
+  </si>
+  <si>
+    <t>Schedule product demo</t>
+  </si>
+  <si>
+    <t>Northstar is evaluating a CRM implementation.</t>
+  </si>
+  <si>
+    <t>Mobile App Project - GreenLeaf</t>
+  </si>
+  <si>
+    <t>Discuss requirements</t>
+  </si>
+  <si>
+    <t>Potential mobile application development project.</t>
+  </si>
+  <si>
+    <t>ERP Upgrade - MetroWorks</t>
+  </si>
+  <si>
+    <t>Share quotation</t>
+  </si>
+  <si>
+    <t>Customer requested an estimate for an ERP upgrade.</t>
+  </si>
+  <si>
+    <t>Cloud Migration - BrightPath</t>
+  </si>
+  <si>
+    <t>Arrange technical call</t>
+  </si>
+  <si>
+    <t>Potential cloud migration services opportunity.</t>
+  </si>
+  <si>
+    <t>E-commerce Platform - UrbanCart</t>
+  </si>
+  <si>
+    <t>Follow up with customer</t>
+  </si>
+  <si>
+    <t>Customer is considering a new e-commerce platform.</t>
+  </si>
+  <si>
+    <t>Analytics Dashboard - DataSpring</t>
+  </si>
+  <si>
+    <t>Prepare sample dashboard</t>
+  </si>
+  <si>
+    <t>Potential reporting and analytics dashboard.</t>
+  </si>
+  <si>
+    <t>IT Support Contract - Oakridge</t>
+  </si>
+  <si>
+    <t>Confirm service scope</t>
+  </si>
+  <si>
+    <t>Potential annual IT support and maintenance contract.</t>
+  </si>
+  <si>
+    <t>Security Assessment - SecureWave</t>
+  </si>
+  <si>
+    <t>Send assessment plan</t>
+  </si>
+  <si>
+    <t>Customer requested details for a security assessment.</t>
+  </si>
+  <si>
+    <t>HR Portal - PeopleFirst</t>
+  </si>
+  <si>
+    <t>Book stakeholder meeting</t>
+  </si>
+  <si>
+    <t>Potential employee self-service portal project.</t>
+  </si>
+  <si>
+    <t>Inventory System - StoreLine</t>
+  </si>
+  <si>
+    <t>Review workflow</t>
+  </si>
+  <si>
+    <t>Potential inventory management solution.</t>
+  </si>
+  <si>
+    <t>Website Maintenance Renewal - PixelWorks</t>
+  </si>
+  <si>
+    <t>Discuss renewal</t>
+  </si>
+  <si>
+    <t>Renewal opportunity for website maintenance services.</t>
+  </si>
+  <si>
+    <t>API Integration - LinkBridge</t>
+  </si>
+  <si>
+    <t>Validate API scope</t>
+  </si>
+  <si>
+    <t>Potential integration between business systems.</t>
+  </si>
+  <si>
+    <t>Customer Support Portal - HelpHub</t>
+  </si>
+  <si>
+    <t>Share prototype</t>
+  </si>
+  <si>
+    <t>Potential customer support portal with ticket tracking.</t>
+  </si>
+  <si>
+    <t>Process Automation - FlowLogic</t>
+  </si>
+  <si>
+    <t>Arrange discovery call</t>
+  </si>
+  <si>
+    <t>Potential automation of repetitive business workflows.</t>
+  </si>
+  <si>
+    <t>Website Redesign - Summit Group</t>
+  </si>
+  <si>
+    <t>Confirm design scope</t>
+  </si>
+  <si>
+    <t>Website redesign opportunity for a growing business.</t>
+  </si>
+  <si>
+    <t>Mobile App Maintenance - AppHarbor</t>
+  </si>
+  <si>
+    <t>Send maintenance plan</t>
+  </si>
+  <si>
+    <t>Potential ongoing mobile app maintenance contract.</t>
+  </si>
+  <si>
+    <t>Database Optimization - CoreData</t>
+  </si>
+  <si>
+    <t>Review database metrics</t>
+  </si>
+  <si>
+    <t>Potential database performance and optimization project.</t>
+  </si>
+  <si>
+    <t>Learning Portal - SkillBridge</t>
+  </si>
+  <si>
+    <t>Arrange requirements workshop</t>
+  </si>
+  <si>
+    <t>Potential online learning portal development.</t>
+  </si>
+  <si>
+    <t>Warehouse Management - CargoFlow</t>
+  </si>
+  <si>
+    <t>Prepare solution outline</t>
+  </si>
+  <si>
+    <t>Potential warehouse management system implementation.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -570,16 +766,37 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -602,11 +819,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -614,6 +840,21 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1743,4 +1984,443 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" s="6">
+        <v>25000</v>
+      </c>
+      <c r="C2" s="7">
+        <v>46341</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E2" s="8">
+        <v>20</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="6">
+        <v>75000</v>
+      </c>
+      <c r="C3" s="7">
+        <v>46346</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="8">
+        <v>35</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B4" s="6">
+        <v>120000</v>
+      </c>
+      <c r="C4" s="7">
+        <v>46361</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="E4" s="8">
+        <v>25</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" s="6">
+        <v>180000</v>
+      </c>
+      <c r="C5" s="7">
+        <v>46368</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" s="8">
+        <v>40</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B6" s="6">
+        <v>95000</v>
+      </c>
+      <c r="C6" s="7">
+        <v>46374</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E6" s="8">
+        <v>30</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="135.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="6">
+        <v>65000</v>
+      </c>
+      <c r="C7" s="7">
+        <v>46378</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E7" s="8">
+        <v>45</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" s="6">
+        <v>55000</v>
+      </c>
+      <c r="C8" s="7">
+        <v>46395</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E8" s="8">
+        <v>15</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B9" s="6">
+        <v>40000</v>
+      </c>
+      <c r="C9" s="7">
+        <v>46402</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E9" s="8">
+        <v>50</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B10" s="6">
+        <v>30000</v>
+      </c>
+      <c r="C10" s="7">
+        <v>46409</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E10" s="8">
+        <v>20</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B11" s="6">
+        <v>85000</v>
+      </c>
+      <c r="C11" s="7">
+        <v>46420</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" s="8">
+        <v>30</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B12" s="6">
+        <v>110000</v>
+      </c>
+      <c r="C12" s="7">
+        <v>46428</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="E12" s="8">
+        <v>35</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B13" s="6">
+        <v>18000</v>
+      </c>
+      <c r="C13" s="7">
+        <v>46436</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E13" s="8">
+        <v>60</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="6">
+        <v>72000</v>
+      </c>
+      <c r="C14" s="7">
+        <v>46443</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E14" s="8">
+        <v>25</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B15" s="6">
+        <v>68000</v>
+      </c>
+      <c r="C15" s="7">
+        <v>46451</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E15" s="8">
+        <v>40</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="B16" s="6">
+        <v>135000</v>
+      </c>
+      <c r="C16" s="7">
+        <v>46461</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E16" s="8">
+        <v>20</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" s="6">
+        <v>32000</v>
+      </c>
+      <c r="C17" s="7">
+        <v>46466</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="8">
+        <v>55</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B18" s="6">
+        <v>28000</v>
+      </c>
+      <c r="C18" s="7">
+        <v>46474</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" s="8">
+        <v>30</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="6">
+        <v>48000</v>
+      </c>
+      <c r="C19" s="7">
+        <v>46481</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="E19" s="8">
+        <v>25</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B20" s="6">
+        <v>92000</v>
+      </c>
+      <c r="C20" s="7">
+        <v>46489</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E20" s="8">
+        <v>40</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="B21" s="6">
+        <v>145000</v>
+      </c>
+      <c r="C21" s="7">
+        <v>46497</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="E21" s="8">
+        <v>35</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>